<commit_message>
Critères : ajout des ancres 1/3/5 pour les 36 critères (à relire)
Trois colonnes ajoutées à la feuille « Critères ». Pour les critères
« Coût et risque », 5 = très coûteux ou risqué. A9 et F4 restent notés
par KC. Aucune autre feuille modifiée.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MHSDJVadf4KXpXCtw8ey2f
</commit_message>
<xml_diff>
--- a/Project - Scoring.xlsx
+++ b/Project - Scoring.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISEZ-MOI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Critères" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identification" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="LISEZ-MOI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Critères" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Identification" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Critères'!$A$4:$H$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Critères'!$A$4:$K$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Identification'!$A$1:$T$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="1" min="1" max="1"/>
@@ -611,6 +611,9 @@
     <col width="16" customWidth="1" style="1" min="6" max="6"/>
     <col width="30" customWidth="1" style="1" min="7" max="7"/>
     <col width="10" customWidth="1" style="1" min="8" max="8"/>
+    <col width="44" customWidth="1" style="1" min="9" max="9"/>
+    <col width="44" customWidth="1" style="1" min="10" max="10"/>
+    <col width="44" customWidth="1" style="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -623,7 +626,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Échelle : 1 à 5 avec des ancres décrites par critère (à rédiger). Pour « Valeur », 5 = excellent. Pour « Coût et risque », 5 = très coûteux ou risqué. Pas de pondération à ce stade. AJOUT = demandé lors de la dernière session.</t>
+          <t>Échelle : 1 à 5 avec des ancres décrites par critère (rédigées, à relire). Pour « Valeur », 5 = excellent. Pour « Coût et risque », 5 = très coûteux ou risqué. Pas de pondération à ce stade. AJOUT = demandé lors de la dernière session.</t>
         </is>
       </c>
     </row>
@@ -668,6 +671,21 @@
           <t>Statut vs v1</t>
         </is>
       </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>Ancre 1</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>Ancre 3</t>
+        </is>
+      </c>
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Ancre 5</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -710,6 +728,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>Aucun lien avec l'assurance non-vie ni la théorie du risque.</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>Assurance non-vie en simple contexte, ou méthode de la filière (GLM, séries temporelles) appliquée hors assurance.</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>Tarification, fréquence-sévérité, provisionnement ou théorie du risque non-vie au cœur du sujet, sur données d'assurance.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -752,6 +785,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>Aucun lien avec les extrêmes, les périls naturels ou la réassurance.</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Risque climatique ou périls naturels abordés sans queues épaisses ni scénarios, ou méthodes d'extrêmes sur un objet non assurantiel.</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>Valeurs extrêmes, copules, modélisation de catastrophes ou assurabilité du risque climatique au cœur du sujet.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -794,6 +842,21 @@
           <t>AJOUT</t>
         </is>
       </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>Aucun lien avec la mortalité, la longévité, l'incapacité ou l'ALM.</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>Un volet vie ou prévoyance parmi d'autres (mortalité en variable annexe, ALM survolé).</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>Mortalité, longévité, incapacité, ALM ou Solvabilité II vie au cœur du sujet. Critère d'exploration.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -836,6 +899,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Aucun lien avec la finance de marché ; mathématiques élémentaires.</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>Finance de marché (taux, actions, crédit) avec séries temporelles ou modèles classiques ; mathématiques peu visibles dans la fiche.</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Modèles stochastiques, dérivés, courbe de taux ou séries financières, avec un niveau mathématique clairement lisible dans la fiche.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -878,6 +956,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Sujet purement académique, sans client ni lecture business.</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Question métier réelle mais mono-sectorielle, ou restitution à un client seulement implicite.</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>Cas business avec restitution à un client et décision à éclairer, dans l'esprit d'un cabinet de stratégie ou de risque.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -920,6 +1013,21 @@
           <t>AJOUT</t>
         </is>
       </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Aucune mission de type actuariat en cabinet.</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>Étude actuarielle ou réglementaire menée en interne chez un assureur ou une banque, ou cabinet sur un sujet non actuariel.</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>Mission type d'un cabinet d'actuariat : modèle, provisionnement, réglementaire, étude pour assureurs ou réassureurs.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -962,6 +1070,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>Aucun lien avec le secteur public, les pays émergents ou l'assurance paramétrique.</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="inlineStr">
+        <is>
+          <t>Institution publique ou question de développement, sans lien direct avec le risque ou l'assurance.</t>
+        </is>
+      </c>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>Assurance paramétrique, risque climatique souverain, pays émergents ou institution internationale, avec lien direct au risque.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1004,6 +1127,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>Méthode ou outil de niche, difficilement réutilisable ailleurs.</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>Deux ou trois compétences standard (Python, ML classique, séries temporelles), réutilisables mais génériques.</t>
+        </is>
+      </c>
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>Plusieurs compétences recherchées dans plusieurs voies (bayésien, survie, spatial, ML, R et Python) réellement pratiquées.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1046,6 +1184,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>Aucun intérêt ; sujet subi. Note donnée par KC, jamais par un agent.</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>Intérêt correct, sans enthousiasme.</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>Vrai intérêt personnel, tenable sur quatre à cinq mois pour KC et le groupe.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1088,6 +1241,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>Organisme inconnu hors de son cercle.</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="inlineStr">
+        <is>
+          <t>Connu dans son secteur ou en France.</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>Marque connue et influente dans plusieurs secteurs, reconnue à l'international.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1130,6 +1298,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>Marque sans poids auprès des réassureurs, cabinets, acteurs quant ou institutions visés.</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>Marque connue d'une partie seulement des cibles.</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>Marque qui compte directement auprès de plusieurs types de cibles (réassureurs, cabinets, quant, institutions).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1172,6 +1355,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>Encadrant introuvable, sans publication ni poste visible.</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>Praticien confirmé ou chercheur avec quelques publications.</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>Chercheur reconnu (publications nombreuses, financement type ERC) ou responsable de premier plan de l'équipe visée.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1214,6 +1412,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>Intitulé long, obscur ou trompeur ; impossible à résumer en une ligne.</t>
+        </is>
+      </c>
+      <c r="J17" s="9" t="inlineStr">
+        <is>
+          <t>Se comprend après relecture, ou lisible seulement pour un spécialiste.</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr">
+        <is>
+          <t>Intitulé immédiatement clair et vendeur auprès d'un recruteur suisse ou américain.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1256,6 +1469,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Aucune perspective de publication ni de citation.</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>Rapport sérieux mais peu publiable en l'état.</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>Publiable ou citable (revue, workshop, preprint), encadrement académique, utile au dossier double diplôme.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1298,6 +1526,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Aucun lien connu entre l'organisme et le recrutement d'étudiants.</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>L'organisme recrute des stagiaires ou des alternants, mais pas via cette équipe ni ce sujet.</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Équipe qui recrute, programme de stage, ou historique d'élèves recrutés après un StatApp.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -1340,6 +1583,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Pas d'accès à des actuaires ou quants ; encadrant peu disponible.</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>Contact avec un praticien capable d'écrire une lettre honnête.</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>Accès direct à des actuaires ou quants seniors ; lettre à fort poids ; introductions probables.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -1382,6 +1640,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>Organisme local, travail uniquement en français.</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>Organisme international ou travail en anglais, sans présence à Zurich ni aux États-Unis.</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>Travail en anglais et organisme présent à Zurich ou aux États-Unis.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -1424,6 +1697,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Pas de récit défendable : problème flou, aucun résultat attendu.</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Problème et méthode clairs, résultat peu chiffrable.</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>Récit complet (problème, méthode, résultat chiffré), racontable en deux minutes.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -1466,6 +1754,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Note 1, ou commentaire déconseillant le sujet.</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>Note 2. Sujet non noté : 3 par défaut, signalé « inconnue » et non pénalisé (à confirmer par KC).</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>Note 3 avec commentaire positif de l'équipe pédagogique.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1508,6 +1811,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Objectif vague ; ni hypothèse de travail ni livrables.</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>Objectif clair, mais hypothèse ou livrables à préciser.</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>Objectif, hypothèse de travail, données et livrables explicitement précisés.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1550,6 +1868,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>Données publiques précisées, accessibles tout de suite, sans NDA.</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>Données annoncées mais accès non confirmé, ou délai d'accès probable.</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>Données non précisées, sous NDA lourd ou à constituer. Risque n°1.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -1592,6 +1925,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>Méthodes hors de tout cours de 1A et 2A.</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>La moitié des méthodes est vue en cours, le reste est à apprendre seul.</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>Méthodes couvertes par les cours de 2A (GLM, séries temporelles, économétrie, ML).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -1634,6 +1982,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>Niveau juste pour un élève de 2A : ni trop dur, ni trop mince.</t>
+        </is>
+      </c>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t>Un peu trop ambitieux ou un peu léger, ajustable avec l'encadrant.</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>Niveau thèse, ou contenu si mince que la note est en danger.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -1676,6 +2039,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>Encadrant injoignable ou peu impliqué ; historique négatif.</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>Encadrement standard, sans information particulière (information faible).</t>
+        </is>
+      </c>
+      <c r="K28" s="9" t="inlineStr">
+        <is>
+          <t>Encadrant réactif, cadre clair, historique d'encadrement d'élèves ENSAE.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -1718,6 +2096,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>Application de méthodes standard, sans démonstration.</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>Modèles classiques mais non triviaux, quelques éléments théoriques.</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>Démonstrations et modèles non triviaux ; fort signal de « raw power ».</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -1760,6 +2153,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>Méthodes déjà maîtrisées en fin de 2A.</t>
+        </is>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>Une méthode nouvelle et significative (survie, bayésien…), le reste est connu.</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>Plusieurs méthodes nouvelles et valorisables (valeurs extrêmes, survie, bayésien, ML moderne, spatial).</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -1802,6 +2210,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>Livrable confidentiel ou interne ; rien à montrer.</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>Rapport en partie montrable ; code non publiable.</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t>Code, outil ou papier montrables publiquement (portfolio, GitHub, preprint).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -1844,6 +2267,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>Sujet attendu, que beaucoup d'élèves choisiront ; label fidèle au contenu.</t>
+        </is>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>Sujet moyennement populaire.</t>
+        </is>
+      </c>
+      <c r="K32" s="9" t="inlineStr">
+        <is>
+          <t>Peu d'élèves le choisiront, ou alpha caché (label moins bon que le contenu).</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
@@ -1886,6 +2324,21 @@
           <t>AJOUT</t>
         </is>
       </c>
+      <c r="I33" s="11" t="inlineStr">
+        <is>
+          <t>Très largement tenable : bien en deçà du temps disponible par personne.</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>Tenable en travaillant normalement, sans marge. Seuils en heures à calibrer avec KC.</t>
+        </is>
+      </c>
+      <c r="K33" s="11" t="inlineStr">
+        <is>
+          <t>Dépasse le temps disponible par personne, même à 4 ou 5 dans le groupe.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -1928,6 +2381,21 @@
           <t>AJOUT</t>
         </is>
       </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>Méthodes et outils déjà connus ; aucune théorie nouvelle.</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>Une méthode ou un outil nouveau à apprendre en quelques semaines.</t>
+        </is>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>Plusieurs méthodes et outils nouveaux ; théorie lourde à maîtriser avant de produire.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -1970,6 +2438,21 @@
           <t>AJOUT</t>
         </is>
       </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>Données propres et prêtes à l'emploi, ou simulées.</t>
+        </is>
+      </c>
+      <c r="J35" s="11" t="inlineStr">
+        <is>
+          <t>Nettoyage et mise en forme significatifs sur une source.</t>
+        </is>
+      </c>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>Collecte, appariement de plusieurs sources et nettoyage lourd avant toute modélisation.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -2012,6 +2495,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I36" s="9" t="inlineStr">
+        <is>
+          <t>Aucun conflit avec les examens ACAS, la candidature double diplôme ni le point d'étape de mars. Note donnée par KC.</t>
+        </is>
+      </c>
+      <c r="J36" s="9" t="inlineStr">
+        <is>
+          <t>Un pic de charge se superpose en partie à ces échéances.</t>
+        </is>
+      </c>
+      <c r="K36" s="9" t="inlineStr">
+        <is>
+          <t>Charge maximale au moment des examens ou des candidatures.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -2054,6 +2552,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I37" s="9" t="inlineStr">
+        <is>
+          <t>Stack connue, calcul léger, aucune dépendance à un tiers.</t>
+        </is>
+      </c>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>Une dépendance (stack inconnue ou données lourdes), contournable.</t>
+        </is>
+      </c>
+      <c r="K37" s="9" t="inlineStr">
+        <is>
+          <t>GPU, données très lourdes ou dépendance critique à un tiers (accès, encadrant).</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -2096,6 +2609,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I38" s="9" t="inlineStr">
+        <is>
+          <t>Se découpe facilement en quatre ou cinq lots indépendants.</t>
+        </is>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>Se découpe en trois lots, avec des dépendances ordonnées.</t>
+        </is>
+      </c>
+      <c r="K38" s="9" t="inlineStr">
+        <is>
+          <t>Travail essentiellement séquentiel ou monolithique ; lots bloquants.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -2138,6 +2666,21 @@
           <t>v1</t>
         </is>
       </c>
+      <c r="I39" s="9" t="inlineStr">
+        <is>
+          <t>Aucune restriction : projet et code citables et publiables.</t>
+        </is>
+      </c>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>Projet citable, mais code ou données non publiables.</t>
+        </is>
+      </c>
+      <c r="K39" s="9" t="inlineStr">
+        <is>
+          <t>Projet non citable et code interdit de publication (NDA strict).</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -2180,6 +2723,21 @@
           <t>AJOUT</t>
         </is>
       </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>Demande probablement faible : très bonnes chances de l'obtenir avec un bon rang de vœu.</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>Demande moyenne.</t>
+        </is>
+      </c>
+      <c r="K40" s="11" t="inlineStr">
+        <is>
+          <t>Très demandé (marque connue, sujet populaire, note 3) ; peu de chances même en vœu 1.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
@@ -2189,7 +2747,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H40"/>
+  <autoFilter ref="A4:K40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>